<commit_message>
Update report generator script
</commit_message>
<xml_diff>
--- a/tests/benchmarks/reporte_omp.xlsx
+++ b/tests/benchmarks/reporte_omp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanb\Documents\GitHub\HPC-Matrix\tests\benchmarks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FAD45E3-9446-42FA-B55A-DAB6EF19936D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DA322C-4603-4492-8B21-B2A4AAE8FA2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2 hilos" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,8 @@
     <sheet name="6 hilos" sheetId="3" r:id="rId3"/>
     <sheet name="8 hilos" sheetId="4" r:id="rId4"/>
     <sheet name="12 hilos" sheetId="5" r:id="rId5"/>
-    <sheet name="16 hilos" sheetId="6" r:id="rId6"/>
-    <sheet name="Scaling  machine1" sheetId="7" r:id="rId7"/>
-    <sheet name="Scaling  machine2" sheetId="8" r:id="rId8"/>
+    <sheet name="Scaling  machine1" sheetId="6" r:id="rId6"/>
+    <sheet name="Scaling  machine2" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="97">
   <si>
     <t>Comparación entre máquinas  |  2 hilos  |  ref: machine1</t>
   </si>
@@ -167,12 +166,6 @@
     <t>machine2  (12 threads)</t>
   </si>
   <si>
-    <t>Comparación entre máquinas  |  16 hilos  |  ref: machine2</t>
-  </si>
-  <si>
-    <t>machine2  (16 threads)</t>
-  </si>
-  <si>
     <t>Strong Scaling  —  machine1</t>
   </si>
   <si>
@@ -185,245 +178,219 @@
     <t>2t</t>
   </si>
   <si>
-    <t>36.9 ms
-1.00x</t>
-  </si>
-  <si>
-    <t>364.0 ms
-1.00x</t>
-  </si>
-  <si>
-    <t>3,161.2 ms
-1.00x</t>
-  </si>
-  <si>
-    <t>40,334.8 ms
-1.00x</t>
-  </si>
-  <si>
-    <t>362,668.5 ms
-1.00x</t>
+    <t>89.5 ms
+1.00x vs 2t</t>
+  </si>
+  <si>
+    <t>713.0 ms
+1.00x vs 2t</t>
+  </si>
+  <si>
+    <t>6,342.7 ms
+1.00x vs 2t</t>
+  </si>
+  <si>
+    <t>74,025.0 ms
+1.00x vs 2t</t>
+  </si>
+  <si>
+    <t>645,378.8 ms
+1.00x vs 2t</t>
   </si>
   <si>
     <t>4t</t>
   </si>
   <si>
     <t>51.9 ms
-0.71x</t>
+1.72x vs 2t</t>
   </si>
   <si>
     <t>433.6 ms
-0.84x</t>
+1.64x vs 2t</t>
   </si>
   <si>
     <t>3,965.3 ms
-0.80x</t>
+1.60x vs 2t</t>
   </si>
   <si>
     <t>41,159.3 ms
-0.98x</t>
+1.80x vs 2t</t>
   </si>
   <si>
     <t>337,686.0 ms
-1.07x</t>
+1.91x vs 2t</t>
   </si>
   <si>
     <t>6t</t>
   </si>
   <si>
     <t>34.3 ms
-1.08x</t>
+2.61x vs 2t</t>
   </si>
   <si>
     <t>293.6 ms
-1.24x</t>
+2.43x vs 2t</t>
   </si>
   <si>
     <t>2,689.6 ms
-1.18x</t>
+2.36x vs 2t</t>
   </si>
   <si>
     <t>27,181.4 ms
-1.48x</t>
+2.72x vs 2t</t>
   </si>
   <si>
     <t>230,366.5 ms
-1.57x</t>
+2.80x vs 2t</t>
   </si>
   <si>
     <t>8t</t>
   </si>
   <si>
     <t>24.0 ms
-1.54x</t>
+3.73x vs 2t</t>
   </si>
   <si>
     <t>202.5 ms
-1.80x</t>
+3.52x vs 2t</t>
   </si>
   <si>
     <t>1,874.1 ms
-1.69x</t>
+3.38x vs 2t</t>
   </si>
   <si>
     <t>19,431.7 ms
-2.08x</t>
+3.81x vs 2t</t>
   </si>
   <si>
     <t>169,600.1 ms
-2.14x</t>
+3.81x vs 2t</t>
   </si>
   <si>
     <t>12t</t>
   </si>
   <si>
     <t>17.3 ms
-2.14x</t>
+5.18x vs 2t</t>
   </si>
   <si>
     <t>148.6 ms
-2.45x</t>
+4.80x vs 2t</t>
   </si>
   <si>
     <t>1,352.1 ms
-2.34x</t>
+4.69x vs 2t</t>
   </si>
   <si>
     <t>12,801.1 ms
-3.15x</t>
+5.78x vs 2t</t>
   </si>
   <si>
     <t>120,316.3 ms
-3.01x</t>
-  </si>
-  <si>
-    <t>16t</t>
-  </si>
-  <si>
-    <t>—</t>
+5.36x vs 2t</t>
   </si>
   <si>
     <t>Strong Scaling  —  machine2</t>
   </si>
   <si>
     <t>250.3 ms
-1.00x</t>
+1.00x vs 2t</t>
   </si>
   <si>
     <t>2,169.1 ms
-1.00x</t>
+1.00x vs 2t</t>
   </si>
   <si>
     <t>21,892.0 ms
-1.00x</t>
+1.00x vs 2t</t>
   </si>
   <si>
     <t>210,194.5 ms
-1.00x</t>
+1.00x vs 2t</t>
   </si>
   <si>
     <t>1,498,333.0 ms
-1.00x</t>
+1.00x vs 2t</t>
   </si>
   <si>
     <t>121.8 ms
-2.05x</t>
+2.05x vs 2t</t>
   </si>
   <si>
     <t>1,080.9 ms
-2.01x</t>
+2.01x vs 2t</t>
   </si>
   <si>
     <t>11,348.9 ms
-1.93x</t>
+1.93x vs 2t</t>
   </si>
   <si>
     <t>118,760.8 ms
-1.77x</t>
+1.77x vs 2t</t>
   </si>
   <si>
     <t>1,077,906.0 ms
-1.39x</t>
+1.39x vs 2t</t>
   </si>
   <si>
     <t>86.3 ms
-2.90x</t>
+2.90x vs 2t</t>
   </si>
   <si>
     <t>736.8 ms
-2.94x</t>
+2.94x vs 2t</t>
   </si>
   <si>
     <t>7,571.7 ms
-2.89x</t>
+2.89x vs 2t</t>
   </si>
   <si>
     <t>76,523.0 ms
-2.75x</t>
+2.75x vs 2t</t>
   </si>
   <si>
     <t>716,666.2 ms
-2.09x</t>
+2.09x vs 2t</t>
   </si>
   <si>
     <t>60.4 ms
-4.14x</t>
+4.14x vs 2t</t>
   </si>
   <si>
     <t>537.5 ms
-4.04x</t>
+4.04x vs 2t</t>
   </si>
   <si>
     <t>5,631.4 ms
-3.89x</t>
+3.89x vs 2t</t>
   </si>
   <si>
     <t>56,015.1 ms
-3.75x</t>
+3.75x vs 2t</t>
   </si>
   <si>
     <t>464,632.1 ms
-3.22x</t>
+3.22x vs 2t</t>
   </si>
   <si>
     <t>45.1 ms
-5.55x</t>
+5.55x vs 2t</t>
   </si>
   <si>
     <t>379.4 ms
-5.72x</t>
+5.72x vs 2t</t>
   </si>
   <si>
     <t>3,775.8 ms
-5.80x</t>
+5.80x vs 2t</t>
   </si>
   <si>
     <t>39,864.3 ms
-5.27x</t>
+5.27x vs 2t</t>
   </si>
   <si>
     <t>335,229.7 ms
-4.47x</t>
-  </si>
-  <si>
-    <t>33.7 ms
-7.44x</t>
-  </si>
-  <si>
-    <t>278.9 ms
-7.78x</t>
-  </si>
-  <si>
-    <t>2,811.9 ms
-7.79x</t>
-  </si>
-  <si>
-    <t>31,465.7 ms
-6.68x</t>
-  </si>
-  <si>
-    <t>260,280.4 ms
-5.76x</t>
+4.47x vs 2t</t>
   </si>
 </sst>
 </file>
@@ -600,7 +567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -656,9 +623,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -755,6 +719,39 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5905500" cy="3429000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -814,6 +811,39 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5905500" cy="3429000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -897,6 +927,39 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5905500" cy="3429000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -956,6 +1019,39 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5905500" cy="3429000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1039,6 +1135,39 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5905500" cy="3429000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1048,10 +1177,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5905500" cy="3429000"/>
+    <xdr:ext cx="6667500" cy="3810000"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
@@ -1077,39 +1206,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="5905500" cy="3429000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 2" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000003000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1119,7 +1215,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="6667500" cy="3810000"/>
@@ -1129,44 +1225,6 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6667500" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1481,7 +1539,7 @@
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
@@ -1492,34 +1550,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -1606,19 +1664,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="4">
-        <v>0</v>
+        <v>105.846</v>
       </c>
       <c r="C8" s="4">
-        <v>0</v>
+        <v>872.83699999999999</v>
       </c>
       <c r="D8" s="4">
-        <v>0</v>
+        <v>7936.7370000000001</v>
       </c>
       <c r="E8" s="4">
-        <v>0</v>
+        <v>83049.823000000004</v>
       </c>
       <c r="F8" s="4">
-        <v>0</v>
+        <v>736640.41399999999</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1626,19 +1684,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="3">
-        <v>0</v>
+        <v>104.82599999999999</v>
       </c>
       <c r="C9" s="3">
-        <v>0</v>
+        <v>871.65099999999995</v>
       </c>
       <c r="D9" s="3">
-        <v>0</v>
+        <v>7930.4949999999999</v>
       </c>
       <c r="E9" s="3">
-        <v>0</v>
+        <v>83118.343999999997</v>
       </c>
       <c r="F9" s="3">
-        <v>0</v>
+        <v>742675.18400000001</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1646,19 +1704,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="4">
-        <v>0</v>
+        <v>105.416</v>
       </c>
       <c r="C10" s="4">
-        <v>0</v>
+        <v>876.75900000000001</v>
       </c>
       <c r="D10" s="4">
-        <v>0</v>
+        <v>7950.4359999999997</v>
       </c>
       <c r="E10" s="4">
-        <v>0</v>
+        <v>85353.119000000006</v>
       </c>
       <c r="F10" s="4">
-        <v>0</v>
+        <v>738207.63</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1666,19 +1724,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="3">
-        <v>0</v>
+        <v>103.81699999999999</v>
       </c>
       <c r="C11" s="3">
-        <v>0</v>
+        <v>868.17499999999995</v>
       </c>
       <c r="D11" s="3">
-        <v>0</v>
+        <v>7997.4309999999996</v>
       </c>
       <c r="E11" s="3">
-        <v>0</v>
+        <v>85381.11</v>
       </c>
       <c r="F11" s="3">
-        <v>0</v>
+        <v>609580.58700000006</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1686,7 +1744,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="4">
-        <v>0</v>
+        <v>106.006</v>
       </c>
       <c r="C12" s="4">
         <v>475.863</v>
@@ -1746,19 +1804,19 @@
         <v>9</v>
       </c>
       <c r="B15" s="6">
-        <v>36.906999999999996</v>
+        <v>89.498000000000005</v>
       </c>
       <c r="C15" s="6">
-        <v>364.00900000000001</v>
+        <v>712.95100000000002</v>
       </c>
       <c r="D15" s="6">
-        <v>3161.194</v>
+        <v>6342.7030000000004</v>
       </c>
       <c r="E15" s="6">
-        <v>40334.794999999998</v>
+        <v>74025.034</v>
       </c>
       <c r="F15" s="6">
-        <v>362668.462</v>
+        <v>645378.84400000004</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1766,19 +1824,19 @@
         <v>10</v>
       </c>
       <c r="B16" s="7">
-        <v>41.268000000000001</v>
+        <v>24.233000000000001</v>
       </c>
       <c r="C16" s="7">
-        <v>329.654</v>
+        <v>193.08099999999999</v>
       </c>
       <c r="D16" s="7">
-        <v>2999.3719999999998</v>
+        <v>2016.1289999999999</v>
       </c>
       <c r="E16" s="7">
-        <v>35615.311000000002</v>
+        <v>15929.295</v>
       </c>
       <c r="F16" s="7">
-        <v>314380.20699999999</v>
+        <v>122163.534</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1786,19 +1844,19 @@
         <v>11</v>
       </c>
       <c r="B17" s="8">
-        <v>111.82</v>
+        <v>27.08</v>
       </c>
       <c r="C17" s="8">
-        <v>90.56</v>
+        <v>27.08</v>
       </c>
       <c r="D17" s="8">
-        <v>94.88</v>
+        <v>31.79</v>
       </c>
       <c r="E17" s="8">
-        <v>88.3</v>
+        <v>21.52</v>
       </c>
       <c r="F17" s="8">
-        <v>86.69</v>
+        <v>18.93</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="6" customHeight="1" x14ac:dyDescent="0.25">
@@ -1810,14 +1868,14 @@
       <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -2100,14 +2158,14 @@
       </c>
     </row>
     <row r="36" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
     </row>
     <row r="37" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
@@ -2152,31 +2210,31 @@
         <v>2</v>
       </c>
       <c r="B38" s="13">
-        <v>36.906999999999996</v>
+        <v>89.498000000000005</v>
       </c>
       <c r="C38" s="14">
         <v>1</v>
       </c>
       <c r="D38" s="13">
-        <v>364.00900000000001</v>
+        <v>712.95100000000002</v>
       </c>
       <c r="E38" s="14">
         <v>1</v>
       </c>
       <c r="F38" s="13">
-        <v>3161.194</v>
+        <v>6342.7030000000004</v>
       </c>
       <c r="G38" s="14">
         <v>1</v>
       </c>
       <c r="H38" s="13">
-        <v>40334.794999999998</v>
+        <v>74025.034</v>
       </c>
       <c r="I38" s="14">
         <v>1</v>
       </c>
       <c r="J38" s="13">
-        <v>362668.462</v>
+        <v>645378.84400000004</v>
       </c>
       <c r="K38" s="14">
         <v>1</v>
@@ -2193,35 +2251,35 @@
         <v>250.25299999999999</v>
       </c>
       <c r="C39" s="14">
-        <v>0.14749999999999999</v>
+        <v>0.35759999999999997</v>
       </c>
       <c r="D39" s="16">
         <v>2169.0859999999998</v>
       </c>
       <c r="E39" s="14">
-        <v>0.1678</v>
+        <v>0.32869999999999999</v>
       </c>
       <c r="F39" s="16">
         <v>21892.008999999998</v>
       </c>
       <c r="G39" s="14">
-        <v>0.1444</v>
+        <v>0.28970000000000001</v>
       </c>
       <c r="H39" s="16">
         <v>210194.519</v>
       </c>
       <c r="I39" s="14">
-        <v>0.19189999999999999</v>
+        <v>0.35220000000000001</v>
       </c>
       <c r="J39" s="16">
         <v>1498332.9790000001</v>
       </c>
       <c r="K39" s="14">
-        <v>0.24199999999999999</v>
+        <v>0.43070000000000003</v>
       </c>
       <c r="L39" s="15">
         <f>IFERROR(AVERAGE(C39,E39,G39,I39,K39),"N/A")</f>
-        <v>0.17871999999999999</v>
+        <v>0.35178000000000004</v>
       </c>
     </row>
   </sheetData>
@@ -2257,34 +2315,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -2575,14 +2633,14 @@
       <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -2865,14 +2923,14 @@
       </c>
     </row>
     <row r="36" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
     </row>
     <row r="37" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
@@ -3022,34 +3080,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -3340,14 +3398,14 @@
       <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -3630,14 +3688,14 @@
       </c>
     </row>
     <row r="36" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
     </row>
     <row r="37" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
@@ -3787,34 +3845,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -4105,14 +4163,14 @@
       <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -4395,14 +4453,14 @@
       </c>
     </row>
     <row r="36" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
     </row>
     <row r="37" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
@@ -4552,34 +4610,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -4870,14 +4928,14 @@
       <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -5160,14 +5218,14 @@
       </c>
     </row>
     <row r="36" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B36" s="22"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
     </row>
     <row r="37" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
@@ -5299,434 +5357,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:L22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-    </row>
-    <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-    </row>
-    <row r="3" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-    </row>
-    <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>1</v>
-      </c>
-      <c r="B5" s="3">
-        <v>33.767000000000003</v>
-      </c>
-      <c r="C5" s="3">
-        <v>278.73200000000003</v>
-      </c>
-      <c r="D5" s="3">
-        <v>2806.8290000000002</v>
-      </c>
-      <c r="E5" s="3">
-        <v>31508.763999999999</v>
-      </c>
-      <c r="F5" s="3">
-        <v>260496.86300000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>2</v>
-      </c>
-      <c r="B6" s="4">
-        <v>33.67</v>
-      </c>
-      <c r="C6" s="4">
-        <v>279.19600000000003</v>
-      </c>
-      <c r="D6" s="4">
-        <v>2807.3409999999999</v>
-      </c>
-      <c r="E6" s="4">
-        <v>31432.047999999999</v>
-      </c>
-      <c r="F6" s="4">
-        <v>261477.171</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3">
-        <v>33.655999999999999</v>
-      </c>
-      <c r="C7" s="3">
-        <v>279.14699999999999</v>
-      </c>
-      <c r="D7" s="3">
-        <v>2812.806</v>
-      </c>
-      <c r="E7" s="3">
-        <v>31697.258000000002</v>
-      </c>
-      <c r="F7" s="3">
-        <v>261147.07699999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4">
-        <v>33.587000000000003</v>
-      </c>
-      <c r="C8" s="4">
-        <v>278.803</v>
-      </c>
-      <c r="D8" s="4">
-        <v>2811.6509999999998</v>
-      </c>
-      <c r="E8" s="4">
-        <v>31295.745999999999</v>
-      </c>
-      <c r="F8" s="4">
-        <v>256784.274</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
-        <v>5</v>
-      </c>
-      <c r="B9" s="3">
-        <v>33.645000000000003</v>
-      </c>
-      <c r="C9" s="3">
-        <v>278.55599999999998</v>
-      </c>
-      <c r="D9" s="3">
-        <v>2795.6680000000001</v>
-      </c>
-      <c r="E9" s="3">
-        <v>31512.300999999999</v>
-      </c>
-      <c r="F9" s="3">
-        <v>259581.23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
-        <v>6</v>
-      </c>
-      <c r="B10" s="4">
-        <v>33.680999999999997</v>
-      </c>
-      <c r="C10" s="4">
-        <v>278.786</v>
-      </c>
-      <c r="D10" s="4">
-        <v>2816.3449999999998</v>
-      </c>
-      <c r="E10" s="4">
-        <v>31410.686000000002</v>
-      </c>
-      <c r="F10" s="4">
-        <v>259342.34899999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
-        <v>7</v>
-      </c>
-      <c r="B11" s="3">
-        <v>33.713999999999999</v>
-      </c>
-      <c r="C11" s="3">
-        <v>279.25099999999998</v>
-      </c>
-      <c r="D11" s="3">
-        <v>2819.9140000000002</v>
-      </c>
-      <c r="E11" s="3">
-        <v>31543.156999999999</v>
-      </c>
-      <c r="F11" s="3">
-        <v>261480.41800000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
-        <v>8</v>
-      </c>
-      <c r="B12" s="4">
-        <v>33.579000000000001</v>
-      </c>
-      <c r="C12" s="4">
-        <v>278.16899999999998</v>
-      </c>
-      <c r="D12" s="4">
-        <v>2809.5749999999998</v>
-      </c>
-      <c r="E12" s="4">
-        <v>31441.05</v>
-      </c>
-      <c r="F12" s="4">
-        <v>262938.8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
-        <v>9</v>
-      </c>
-      <c r="B13" s="3">
-        <v>33.597000000000001</v>
-      </c>
-      <c r="C13" s="3">
-        <v>279.54899999999998</v>
-      </c>
-      <c r="D13" s="3">
-        <v>2836.7559999999999</v>
-      </c>
-      <c r="E13" s="3">
-        <v>31603.453000000001</v>
-      </c>
-      <c r="F13" s="3">
-        <v>260020.99900000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
-        <v>10</v>
-      </c>
-      <c r="B14" s="4">
-        <v>33.610999999999997</v>
-      </c>
-      <c r="C14" s="4">
-        <v>278.89999999999998</v>
-      </c>
-      <c r="D14" s="4">
-        <v>2801.69</v>
-      </c>
-      <c r="E14" s="4">
-        <v>31212.402999999998</v>
-      </c>
-      <c r="F14" s="4">
-        <v>259534.33600000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" s="6">
-        <v>33.651000000000003</v>
-      </c>
-      <c r="C15" s="6">
-        <v>278.90899999999999</v>
-      </c>
-      <c r="D15" s="6">
-        <v>2811.8580000000002</v>
-      </c>
-      <c r="E15" s="6">
-        <v>31465.687000000002</v>
-      </c>
-      <c r="F15" s="6">
-        <v>260280.35200000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16" s="7">
-        <v>5.7000000000000002E-2</v>
-      </c>
-      <c r="C16" s="7">
-        <v>0.374</v>
-      </c>
-      <c r="D16" s="7">
-        <v>10.593999999999999</v>
-      </c>
-      <c r="E16" s="7">
-        <v>134.32499999999999</v>
-      </c>
-      <c r="F16" s="7">
-        <v>1579.65</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="8">
-        <v>0.17</v>
-      </c>
-      <c r="C17" s="8">
-        <v>0.13</v>
-      </c>
-      <c r="D17" s="8">
-        <v>0.38</v>
-      </c>
-      <c r="E17" s="8">
-        <v>0.43</v>
-      </c>
-      <c r="F17" s="8">
-        <v>0.61</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-    </row>
-    <row r="21" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L21" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="B22" s="13">
-        <v>33.651000000000003</v>
-      </c>
-      <c r="C22" s="14">
-        <v>1</v>
-      </c>
-      <c r="D22" s="13">
-        <v>278.90899999999999</v>
-      </c>
-      <c r="E22" s="14">
-        <v>1</v>
-      </c>
-      <c r="F22" s="13">
-        <v>2811.8580000000002</v>
-      </c>
-      <c r="G22" s="14">
-        <v>1</v>
-      </c>
-      <c r="H22" s="13">
-        <v>31465.687000000002</v>
-      </c>
-      <c r="I22" s="14">
-        <v>1</v>
-      </c>
-      <c r="J22" s="13">
-        <v>260280.35200000001</v>
-      </c>
-      <c r="K22" s="14">
-        <v>1</v>
-      </c>
-      <c r="L22" s="15">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5735,28 +5366,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="A1" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="A2" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>4</v>
@@ -5776,122 +5407,102 @@
     </row>
     <row r="4" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="D4" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="E4" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="F4" s="18" t="s">
         <v>46</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="D5" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="E5" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="F5" s="19" t="s">
         <v>52</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="D6" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="E6" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="F6" s="18" t="s">
         <v>58</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="D7" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="E7" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="F7" s="19" t="s">
         <v>64</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="D8" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="F8" s="18" t="s">
         <v>70</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -5904,9 +5515,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:F9"/>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5915,28 +5526,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="A1" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="A2" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>4</v>
@@ -5956,122 +5567,102 @@
     </row>
     <row r="4" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B4" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="18" t="s">
         <v>76</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="E4" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B5" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="F5" s="19" t="s">
         <v>81</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B6" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="F6" s="18" t="s">
         <v>86</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B7" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="F7" s="19" t="s">
         <v>91</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="E7" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B8" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F8" s="18" t="s">
         <v>96</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>103</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added strong scaling tables and corrected tipografy errors
</commit_message>
<xml_diff>
--- a/tests/benchmarks/reporte_omp.xlsx
+++ b/tests/benchmarks/reporte_omp.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DA322C-4603-4492-8B21-B2A4AAE8FA2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2 hilos" sheetId="1" r:id="rId1"/>

</xml_diff>